<commit_message>
Added new tables and imported data
</commit_message>
<xml_diff>
--- a/data/nfl/nfl_currentTeams.xlsx
+++ b/data/nfl/nfl_currentTeams.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shawn\Documents\sportsdataappgroupproject1-bhss\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GroupProjectFolder\sportsdataappgroupproject1-bhss\data\nfl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D8EF6F06-5724-4BE9-AFDC-0BA87F2A15B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4C10AE2-F871-48AD-8697-B2DEE1E44616}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{85773CD1-30A4-40A8-B24B-AF12438DAEFA}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{85773CD1-30A4-40A8-B24B-AF12438DAEFA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="100">
   <si>
     <t>Arizona Cardinals</t>
   </si>
@@ -134,19 +134,208 @@
     <t>Seattle Seahawks</t>
   </si>
   <si>
-    <t>TeamId</t>
-  </si>
-  <si>
     <t>Name</t>
   </si>
   <si>
-    <t>Wins</t>
-  </si>
-  <si>
-    <t>Losses</t>
-  </si>
-  <si>
-    <t>Ties</t>
+    <t>abr</t>
+  </si>
+  <si>
+    <t>conf</t>
+  </si>
+  <si>
+    <t>stadium</t>
+  </si>
+  <si>
+    <t>ARI</t>
+  </si>
+  <si>
+    <t>ATL</t>
+  </si>
+  <si>
+    <t>BAL</t>
+  </si>
+  <si>
+    <t>BUF</t>
+  </si>
+  <si>
+    <t>CAR</t>
+  </si>
+  <si>
+    <t>CHI</t>
+  </si>
+  <si>
+    <t>CIN</t>
+  </si>
+  <si>
+    <t>CLE</t>
+  </si>
+  <si>
+    <t>DAL</t>
+  </si>
+  <si>
+    <t>DEN</t>
+  </si>
+  <si>
+    <t>DET</t>
+  </si>
+  <si>
+    <t>GB</t>
+  </si>
+  <si>
+    <t>HOU</t>
+  </si>
+  <si>
+    <t>IND</t>
+  </si>
+  <si>
+    <t>JAX</t>
+  </si>
+  <si>
+    <t>KC</t>
+  </si>
+  <si>
+    <t>LV</t>
+  </si>
+  <si>
+    <t>LAC</t>
+  </si>
+  <si>
+    <t>LAR</t>
+  </si>
+  <si>
+    <t>MIA</t>
+  </si>
+  <si>
+    <t>MIN</t>
+  </si>
+  <si>
+    <t>NE</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
+    <t>NYG</t>
+  </si>
+  <si>
+    <t>NYJ</t>
+  </si>
+  <si>
+    <t>PHI</t>
+  </si>
+  <si>
+    <t>PIT</t>
+  </si>
+  <si>
+    <t>SF</t>
+  </si>
+  <si>
+    <t>SEA</t>
+  </si>
+  <si>
+    <t>TB</t>
+  </si>
+  <si>
+    <t>TEN</t>
+  </si>
+  <si>
+    <t>WAS</t>
+  </si>
+  <si>
+    <t>NFC</t>
+  </si>
+  <si>
+    <t>AFC</t>
+  </si>
+  <si>
+    <t>State Farm Stadium</t>
+  </si>
+  <si>
+    <t>Mercedes-Benz Stadium</t>
+  </si>
+  <si>
+    <t>M&amp;T Bank Stadium</t>
+  </si>
+  <si>
+    <t>Highmark Stadium</t>
+  </si>
+  <si>
+    <t>Bank of America Stadium</t>
+  </si>
+  <si>
+    <t>Soldier Field</t>
+  </si>
+  <si>
+    <t>Paycor Stadium</t>
+  </si>
+  <si>
+    <t>Huntington Bank Field</t>
+  </si>
+  <si>
+    <t>AT&amp;T Stadium</t>
+  </si>
+  <si>
+    <t>Empower Field at Mile High</t>
+  </si>
+  <si>
+    <t>Ford Field</t>
+  </si>
+  <si>
+    <t>Lambeau Field</t>
+  </si>
+  <si>
+    <t>NRG Stadium</t>
+  </si>
+  <si>
+    <t>Lucas Oil Stadium</t>
+  </si>
+  <si>
+    <t>EverBank Stadium</t>
+  </si>
+  <si>
+    <t>GEHA Field at Arrowhead Stadium</t>
+  </si>
+  <si>
+    <t>Allegiant Stadium</t>
+  </si>
+  <si>
+    <t>SoFi Stadium</t>
+  </si>
+  <si>
+    <t>Hard Rock Stadium</t>
+  </si>
+  <si>
+    <t>U.S. Bank Stadium</t>
+  </si>
+  <si>
+    <t>Gillette Stadium</t>
+  </si>
+  <si>
+    <t>Caesars Superdome</t>
+  </si>
+  <si>
+    <t>MetLife Stadium</t>
+  </si>
+  <si>
+    <t>Lincoln Financial Field</t>
+  </si>
+  <si>
+    <t>Acrisure Stadium</t>
+  </si>
+  <si>
+    <t>Levi's Stadium</t>
+  </si>
+  <si>
+    <t>Lumen Field</t>
+  </si>
+  <si>
+    <t>Raymond James Stadium</t>
+  </si>
+  <si>
+    <t>Nissan Stadium</t>
+  </si>
+  <si>
+    <t>Northwest Stadium</t>
   </si>
 </sst>
 </file>
@@ -182,9 +371,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -206,13 +394,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
@@ -255,13 +443,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
@@ -304,13 +492,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
@@ -353,13 +541,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
@@ -402,13 +590,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>6</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
@@ -451,13 +639,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>6</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
@@ -500,13 +688,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>8</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
@@ -549,13 +737,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>8</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>9</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
@@ -598,13 +786,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>9</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>10</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
@@ -647,13 +835,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>10</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>11</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
@@ -696,13 +884,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>11</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>12</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
@@ -745,13 +933,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>12</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>13</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
@@ -794,13 +982,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>13</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
@@ -843,13 +1031,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>15</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
@@ -892,13 +1080,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>15</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>16</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
@@ -941,13 +1129,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>16</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>17</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
@@ -990,13 +1178,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>17</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>18</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
@@ -1039,13 +1227,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>18</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>19</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
@@ -1088,13 +1276,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>19</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>20</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
@@ -1137,13 +1325,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>20</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
@@ -1186,13 +1374,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>22</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
@@ -1235,13 +1423,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>22</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>23</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
@@ -1284,13 +1472,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>23</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>24</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
@@ -1333,13 +1521,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>24</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>25</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
@@ -1382,13 +1570,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>25</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>26</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
@@ -1431,13 +1619,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>26</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>27</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
@@ -1480,13 +1668,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>27</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>28</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
@@ -1529,13 +1717,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>28</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>29</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
@@ -1578,13 +1766,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>29</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>30</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
@@ -1627,13 +1815,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>30</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>31</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
@@ -1676,13 +1864,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>31</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>32</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
@@ -1725,13 +1913,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>32</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>33</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
@@ -2092,14 +2280,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68A7C8D9-0054-4E51-B7E1-A82891079390}">
-  <dimension ref="A1:E33"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D33"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="25.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.28515625" customWidth="1"/>
+    <col min="1" max="1" width="25.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>32</v>
       </c>
@@ -2112,552 +2300,453 @@
       <c r="D1" t="s">
         <v>35</v>
       </c>
-      <c r="E1" t="s">
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2">
+      <c r="C2" t="s">
+        <v>68</v>
+      </c>
+      <c r="D2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2">
+      <c r="B3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C3" t="s">
+        <v>68</v>
+      </c>
+      <c r="D3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4" t="s">
+        <v>69</v>
+      </c>
+      <c r="D4" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>3</v>
       </c>
-      <c r="D2">
+      <c r="B5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C5" t="s">
+        <v>69</v>
+      </c>
+      <c r="D5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C6" t="s">
+        <v>68</v>
+      </c>
+      <c r="D6" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" t="s">
+        <v>68</v>
+      </c>
+      <c r="D7" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" t="s">
+        <v>69</v>
+      </c>
+      <c r="D8" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9" t="s">
+        <v>43</v>
+      </c>
+      <c r="C9" t="s">
+        <v>69</v>
+      </c>
+      <c r="D9" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10" t="s">
+        <v>68</v>
+      </c>
+      <c r="D10" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11" t="s">
+        <v>45</v>
+      </c>
+      <c r="C11" t="s">
+        <v>69</v>
+      </c>
+      <c r="D11" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>7</v>
+      </c>
+      <c r="B12" t="s">
+        <v>46</v>
+      </c>
+      <c r="C12" t="s">
+        <v>68</v>
+      </c>
+      <c r="D12" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>22</v>
+      </c>
+      <c r="B13" t="s">
+        <v>47</v>
+      </c>
+      <c r="C13" t="s">
+        <v>68</v>
+      </c>
+      <c r="D13" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>23</v>
+      </c>
+      <c r="B14" t="s">
+        <v>48</v>
+      </c>
+      <c r="C14" t="s">
+        <v>69</v>
+      </c>
+      <c r="D14" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>8</v>
+      </c>
+      <c r="B15" t="s">
+        <v>49</v>
+      </c>
+      <c r="C15" t="s">
+        <v>69</v>
+      </c>
+      <c r="D15" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16" t="s">
+        <v>50</v>
+      </c>
+      <c r="C16" t="s">
+        <v>69</v>
+      </c>
+      <c r="D16" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>9</v>
+      </c>
+      <c r="B17" t="s">
+        <v>51</v>
+      </c>
+      <c r="C17" t="s">
+        <v>69</v>
+      </c>
+      <c r="D17" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>10</v>
+      </c>
+      <c r="B18" t="s">
+        <v>52</v>
+      </c>
+      <c r="C18" t="s">
+        <v>69</v>
+      </c>
+      <c r="D18" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>25</v>
+      </c>
+      <c r="B19" t="s">
+        <v>53</v>
+      </c>
+      <c r="C19" t="s">
+        <v>69</v>
+      </c>
+      <c r="D19" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20" t="s">
+        <v>54</v>
+      </c>
+      <c r="C20" t="s">
+        <v>68</v>
+      </c>
+      <c r="D20" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>11</v>
+      </c>
+      <c r="B21" t="s">
+        <v>55</v>
+      </c>
+      <c r="C21" t="s">
+        <v>69</v>
+      </c>
+      <c r="D21" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>12</v>
+      </c>
+      <c r="B22" t="s">
+        <v>56</v>
+      </c>
+      <c r="C22" t="s">
+        <v>68</v>
+      </c>
+      <c r="D22" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>27</v>
+      </c>
+      <c r="B23" t="s">
+        <v>57</v>
+      </c>
+      <c r="C23" t="s">
+        <v>69</v>
+      </c>
+      <c r="D23" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>13</v>
+      </c>
+      <c r="B24" t="s">
+        <v>58</v>
+      </c>
+      <c r="C24" t="s">
+        <v>68</v>
+      </c>
+      <c r="D24" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
         <v>14</v>
       </c>
-      <c r="E2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3">
-        <v>8</v>
-      </c>
-      <c r="D3">
-        <v>9</v>
-      </c>
-      <c r="E3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C4">
-        <v>8</v>
-      </c>
-      <c r="D4">
-        <v>9</v>
-      </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C5">
-        <v>12</v>
-      </c>
-      <c r="D5">
-        <v>5</v>
-      </c>
-      <c r="E5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C6">
-        <v>8</v>
-      </c>
-      <c r="D6">
-        <v>9</v>
-      </c>
-      <c r="E6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C7">
-        <v>11</v>
-      </c>
-      <c r="D7">
-        <v>6</v>
-      </c>
-      <c r="E7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C8">
-        <v>6</v>
-      </c>
-      <c r="D8">
-        <v>11</v>
-      </c>
-      <c r="E8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C9">
-        <v>5</v>
-      </c>
-      <c r="D9">
-        <v>12</v>
-      </c>
-      <c r="E9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C10">
-        <v>7</v>
-      </c>
-      <c r="D10">
-        <v>9</v>
-      </c>
-      <c r="E10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C11">
-        <v>14</v>
-      </c>
-      <c r="D11">
-        <v>3</v>
-      </c>
-      <c r="E11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C12">
-        <v>9</v>
-      </c>
-      <c r="D12">
-        <v>8</v>
-      </c>
-      <c r="E12">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13">
-        <v>12</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C13">
-        <v>9</v>
-      </c>
-      <c r="D13">
-        <v>7</v>
-      </c>
-      <c r="E13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14">
-        <v>13</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C14">
-        <v>12</v>
-      </c>
-      <c r="D14">
-        <v>5</v>
-      </c>
-      <c r="E14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15">
-        <v>14</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C15">
-        <v>8</v>
-      </c>
-      <c r="D15">
-        <v>9</v>
-      </c>
-      <c r="E15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16">
+      <c r="B25" t="s">
+        <v>59</v>
+      </c>
+      <c r="C25" t="s">
+        <v>68</v>
+      </c>
+      <c r="D25" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="C16">
-        <v>13</v>
-      </c>
-      <c r="D16">
-        <v>4</v>
-      </c>
-      <c r="E16">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17">
+      <c r="B26" t="s">
+        <v>60</v>
+      </c>
+      <c r="C26" t="s">
+        <v>69</v>
+      </c>
+      <c r="D26" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>28</v>
+      </c>
+      <c r="B27" t="s">
+        <v>61</v>
+      </c>
+      <c r="C27" t="s">
+        <v>68</v>
+      </c>
+      <c r="D27" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>29</v>
+      </c>
+      <c r="B28" t="s">
+        <v>62</v>
+      </c>
+      <c r="C28" t="s">
+        <v>69</v>
+      </c>
+      <c r="D28" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>30</v>
+      </c>
+      <c r="B29" t="s">
+        <v>63</v>
+      </c>
+      <c r="C29" t="s">
+        <v>68</v>
+      </c>
+      <c r="D29" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>31</v>
+      </c>
+      <c r="B30" t="s">
+        <v>64</v>
+      </c>
+      <c r="C30" t="s">
+        <v>68</v>
+      </c>
+      <c r="D30" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
         <v>16</v>
       </c>
-      <c r="B17" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C17">
-        <v>6</v>
-      </c>
-      <c r="D17">
-        <v>11</v>
-      </c>
-      <c r="E17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18">
+      <c r="B31" t="s">
+        <v>65</v>
+      </c>
+      <c r="C31" t="s">
+        <v>68</v>
+      </c>
+      <c r="D31" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
         <v>17</v>
       </c>
-      <c r="B18" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C18">
-        <v>3</v>
-      </c>
-      <c r="D18">
-        <v>14</v>
-      </c>
-      <c r="E18">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19">
+      <c r="B32" t="s">
+        <v>66</v>
+      </c>
+      <c r="C32" t="s">
+        <v>69</v>
+      </c>
+      <c r="D32" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
         <v>18</v>
       </c>
-      <c r="B19" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C19">
-        <v>11</v>
-      </c>
-      <c r="D19">
-        <v>6</v>
-      </c>
-      <c r="E19">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20">
-        <v>19</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C20">
-        <v>12</v>
-      </c>
-      <c r="D20">
-        <v>5</v>
-      </c>
-      <c r="E20">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21">
-        <v>20</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C21">
-        <v>7</v>
-      </c>
-      <c r="D21">
-        <v>10</v>
-      </c>
-      <c r="E21">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22">
-        <v>21</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C22">
-        <v>9</v>
-      </c>
-      <c r="D22">
-        <v>8</v>
-      </c>
-      <c r="E22">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23">
-        <v>22</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="C23">
-        <v>14</v>
-      </c>
-      <c r="D23">
-        <v>3</v>
-      </c>
-      <c r="E23">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24">
-        <v>23</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C24">
-        <v>6</v>
-      </c>
-      <c r="D24">
-        <v>11</v>
-      </c>
-      <c r="E24">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25">
-        <v>24</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C25">
-        <v>4</v>
-      </c>
-      <c r="D25">
-        <v>13</v>
-      </c>
-      <c r="E25">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26">
-        <v>25</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C26">
-        <v>3</v>
-      </c>
-      <c r="D26">
-        <v>14</v>
-      </c>
-      <c r="E26">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27">
-        <v>26</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C27">
-        <v>11</v>
-      </c>
-      <c r="D27">
-        <v>6</v>
-      </c>
-      <c r="E27">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28">
-        <v>27</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C28">
-        <v>10</v>
-      </c>
-      <c r="D28">
-        <v>7</v>
-      </c>
-      <c r="E28">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29">
-        <v>28</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C29">
-        <v>12</v>
-      </c>
-      <c r="D29">
-        <v>5</v>
-      </c>
-      <c r="E29">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30">
-        <v>29</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C30">
-        <v>14</v>
-      </c>
-      <c r="D30">
-        <v>3</v>
-      </c>
-      <c r="E30">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31">
-        <v>30</v>
-      </c>
-      <c r="B31" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C31">
-        <v>8</v>
-      </c>
-      <c r="D31">
-        <v>9</v>
-      </c>
-      <c r="E31">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32">
-        <v>31</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C32">
-        <v>3</v>
-      </c>
-      <c r="D32">
-        <v>14</v>
-      </c>
-      <c r="E32">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33">
-        <v>32</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C33">
-        <v>5</v>
-      </c>
-      <c r="D33">
-        <v>12</v>
-      </c>
-      <c r="E33">
-        <v>0</v>
+      <c r="B33" t="s">
+        <v>67</v>
+      </c>
+      <c r="C33" t="s">
+        <v>68</v>
+      </c>
+      <c r="D33" t="s">
+        <v>99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>